<commit_message>
update the Code of Question One
</commit_message>
<xml_diff>
--- a/Question_One/result1_question_one.xlsx
+++ b/Question_One/result1_question_one.xlsx
@@ -824,7 +824,7 @@
         </is>
       </c>
       <c r="B37" s="7" t="n">
-        <v>2.2539</v>
+        <v>0</v>
       </c>
     </row>
     <row r="38" ht="14" customHeight="1">
@@ -844,7 +844,7 @@
         </is>
       </c>
       <c r="B39" s="7" t="n">
-        <v>4.504</v>
+        <v>0</v>
       </c>
     </row>
     <row r="40" ht="14" customHeight="1">
@@ -894,7 +894,7 @@
         </is>
       </c>
       <c r="B44" s="7" t="n">
-        <v>5.4436</v>
+        <v>0</v>
       </c>
     </row>
     <row r="45" ht="14" customHeight="1">
@@ -904,7 +904,7 @@
         </is>
       </c>
       <c r="B45" s="7" t="n">
-        <v>5.0667</v>
+        <v>0</v>
       </c>
     </row>
     <row r="46" ht="14" customHeight="1">
@@ -914,7 +914,7 @@
         </is>
       </c>
       <c r="B46" s="7" t="n">
-        <v>5.9968</v>
+        <v>0</v>
       </c>
     </row>
     <row r="47" ht="14" customHeight="1">
@@ -924,7 +924,7 @@
         </is>
       </c>
       <c r="B47" s="7" t="n">
-        <v>4.3636</v>
+        <v>0</v>
       </c>
     </row>
     <row r="48" ht="14" customHeight="1">
@@ -934,7 +934,7 @@
         </is>
       </c>
       <c r="B48" s="7" t="n">
-        <v>5.6841</v>
+        <v>0</v>
       </c>
     </row>
     <row r="49" ht="14" customHeight="1">
@@ -944,7 +944,7 @@
         </is>
       </c>
       <c r="B49" s="7" t="n">
-        <v>4.4214</v>
+        <v>0</v>
       </c>
     </row>
     <row r="50" ht="14" customHeight="1">
@@ -954,7 +954,7 @@
         </is>
       </c>
       <c r="B50" s="7" t="n">
-        <v>3.9108</v>
+        <v>0</v>
       </c>
     </row>
     <row r="51" ht="14" customHeight="1">
@@ -964,7 +964,7 @@
         </is>
       </c>
       <c r="B51" s="7" t="n">
-        <v>3.5563</v>
+        <v>0</v>
       </c>
     </row>
     <row r="52" ht="14" customHeight="1">
@@ -974,7 +974,7 @@
         </is>
       </c>
       <c r="B52" s="7" t="n">
-        <v>3.6194</v>
+        <v>0</v>
       </c>
     </row>
     <row r="53" ht="14" customHeight="1">
@@ -1004,7 +1004,7 @@
         </is>
       </c>
       <c r="B55" s="7" t="n">
-        <v>2.3921</v>
+        <v>0</v>
       </c>
     </row>
     <row r="56" ht="14" customHeight="1">
@@ -1014,7 +1014,7 @@
         </is>
       </c>
       <c r="B56" s="7" t="n">
-        <v>4.2595</v>
+        <v>0</v>
       </c>
     </row>
     <row r="57" ht="14" customHeight="1">
@@ -1024,7 +1024,7 @@
         </is>
       </c>
       <c r="B57" s="7" t="n">
-        <v>1.3969</v>
+        <v>0</v>
       </c>
     </row>
     <row r="58" ht="14" customHeight="1">
@@ -1034,7 +1034,7 @@
         </is>
       </c>
       <c r="B58" s="7" t="n">
-        <v>4.5622</v>
+        <v>0</v>
       </c>
     </row>
     <row r="59" ht="14" customHeight="1">
@@ -1044,7 +1044,7 @@
         </is>
       </c>
       <c r="B59" s="7" t="n">
-        <v>4.7982</v>
+        <v>0</v>
       </c>
     </row>
     <row r="60" ht="14" customHeight="1">
@@ -1054,7 +1054,7 @@
         </is>
       </c>
       <c r="B60" s="7" t="n">
-        <v>2.7178</v>
+        <v>0</v>
       </c>
     </row>
     <row r="61" ht="14" customHeight="1">
@@ -1064,7 +1064,7 @@
         </is>
       </c>
       <c r="B61" s="7" t="n">
-        <v>4.3265</v>
+        <v>0</v>
       </c>
     </row>
     <row r="62" ht="14" customHeight="1">
@@ -1074,7 +1074,7 @@
         </is>
       </c>
       <c r="B62" s="7" t="n">
-        <v>5.2386</v>
+        <v>0</v>
       </c>
     </row>
     <row r="63" ht="14" customHeight="1">
@@ -1094,7 +1094,7 @@
         </is>
       </c>
       <c r="B64" s="7" t="n">
-        <v>4.2575</v>
+        <v>0</v>
       </c>
     </row>
     <row r="65" ht="14" customHeight="1">
@@ -1124,7 +1124,7 @@
         </is>
       </c>
       <c r="B67" s="7" t="n">
-        <v>0.4352</v>
+        <v>0</v>
       </c>
     </row>
     <row r="68" ht="14" customHeight="1">
@@ -1144,7 +1144,7 @@
         </is>
       </c>
       <c r="B69" s="7" t="n">
-        <v>5.1462</v>
+        <v>0</v>
       </c>
     </row>
     <row r="70" ht="14" customHeight="1">
@@ -1154,7 +1154,7 @@
         </is>
       </c>
       <c r="B70" s="7" t="n">
-        <v>4.5679</v>
+        <v>0</v>
       </c>
     </row>
     <row r="71" ht="14" customHeight="1">
@@ -1164,7 +1164,7 @@
         </is>
       </c>
       <c r="B71" s="7" t="n">
-        <v>77.3652</v>
+        <v>179.2772</v>
       </c>
     </row>
     <row r="72" ht="14" customHeight="1">
@@ -1194,7 +1194,7 @@
         </is>
       </c>
       <c r="B74" s="7" t="n">
-        <v>480.4125</v>
+        <v>480.4124</v>
       </c>
     </row>
     <row r="75" ht="14" customHeight="1">
@@ -1234,7 +1234,7 @@
         </is>
       </c>
       <c r="B78" s="7" t="n">
-        <v>6.5593</v>
+        <v>0</v>
       </c>
     </row>
     <row r="79" ht="14" customHeight="1">
@@ -1244,7 +1244,7 @@
         </is>
       </c>
       <c r="B79" s="7" t="n">
-        <v>2.1595</v>
+        <v>0</v>
       </c>
     </row>
     <row r="80" ht="14" customHeight="1">
@@ -1254,7 +1254,7 @@
         </is>
       </c>
       <c r="B80" s="7" t="n">
-        <v>1.9369</v>
+        <v>0</v>
       </c>
     </row>
     <row r="81" ht="14" customHeight="1">
@@ -1274,7 +1274,7 @@
         </is>
       </c>
       <c r="B82" s="7" t="n">
-        <v>1.2407</v>
+        <v>0</v>
       </c>
     </row>
     <row r="83" ht="14" customHeight="1">
@@ -1284,7 +1284,7 @@
         </is>
       </c>
       <c r="B83" s="7" t="n">
-        <v>0.418</v>
+        <v>0</v>
       </c>
     </row>
     <row r="84" ht="14" customHeight="1">
@@ -1294,7 +1294,7 @@
         </is>
       </c>
       <c r="B84" s="7" t="n">
-        <v>3.8153</v>
+        <v>0</v>
       </c>
     </row>
     <row r="85" ht="14" customHeight="1">
@@ -1304,7 +1304,7 @@
         </is>
       </c>
       <c r="B85" s="7" t="n">
-        <v>2.1872</v>
+        <v>0</v>
       </c>
     </row>
     <row r="86" ht="14" customHeight="1">
@@ -1314,7 +1314,7 @@
         </is>
       </c>
       <c r="B86" s="7" t="n">
-        <v>1.0744</v>
+        <v>0</v>
       </c>
     </row>
     <row r="87" ht="14" customHeight="1">
@@ -1324,7 +1324,7 @@
         </is>
       </c>
       <c r="B87" s="7" t="n">
-        <v>1.9307</v>
+        <v>0</v>
       </c>
     </row>
     <row r="88" ht="14" customHeight="1">
@@ -1344,7 +1344,7 @@
         </is>
       </c>
       <c r="B89" s="7" t="n">
-        <v>5.7814</v>
+        <v>0</v>
       </c>
     </row>
     <row r="90" ht="14" customHeight="1">
@@ -1354,7 +1354,7 @@
         </is>
       </c>
       <c r="B90" s="7" t="n">
-        <v>4.32</v>
+        <v>0</v>
       </c>
     </row>
     <row r="91" ht="14" customHeight="1">
@@ -1374,7 +1374,7 @@
         </is>
       </c>
       <c r="B92" s="7" t="n">
-        <v>254.2618</v>
+        <v>266.7327</v>
       </c>
     </row>
     <row r="93" ht="14" customHeight="1">
@@ -1554,7 +1554,7 @@
         </is>
       </c>
       <c r="B110" s="7" t="n">
-        <v>101.1613</v>
+        <v>531.894</v>
       </c>
     </row>
     <row r="111" ht="14" customHeight="1">
@@ -1594,7 +1594,7 @@
         </is>
       </c>
       <c r="B114" s="7" t="n">
-        <v>29.6343</v>
+        <v>0</v>
       </c>
     </row>
     <row r="115" ht="14" customHeight="1">
@@ -1604,7 +1604,7 @@
         </is>
       </c>
       <c r="B115" s="7" t="n">
-        <v>31.484</v>
+        <v>0</v>
       </c>
     </row>
     <row r="116" ht="14" customHeight="1">
@@ -1614,7 +1614,7 @@
         </is>
       </c>
       <c r="B116" s="7" t="n">
-        <v>32.4065</v>
+        <v>0</v>
       </c>
     </row>
     <row r="117" ht="14" customHeight="1">
@@ -1624,7 +1624,7 @@
         </is>
       </c>
       <c r="B117" s="7" t="n">
-        <v>33.553</v>
+        <v>0</v>
       </c>
     </row>
     <row r="118" ht="14" customHeight="1">
@@ -1634,7 +1634,7 @@
         </is>
       </c>
       <c r="B118" s="7" t="n">
-        <v>34.4469</v>
+        <v>0</v>
       </c>
     </row>
     <row r="119" ht="14" customHeight="1">
@@ -1644,7 +1644,7 @@
         </is>
       </c>
       <c r="B119" s="7" t="n">
-        <v>36.2324</v>
+        <v>0</v>
       </c>
     </row>
     <row r="120" ht="14" customHeight="1">
@@ -1654,7 +1654,7 @@
         </is>
       </c>
       <c r="B120" s="7" t="n">
-        <v>36.6625</v>
+        <v>0</v>
       </c>
     </row>
     <row r="121" ht="14" customHeight="1">
@@ -1664,7 +1664,7 @@
         </is>
       </c>
       <c r="B121" s="7" t="n">
-        <v>36.445</v>
+        <v>0</v>
       </c>
     </row>
     <row r="122" ht="14" customHeight="1">
@@ -1674,7 +1674,7 @@
         </is>
       </c>
       <c r="B122" s="7" t="n">
-        <v>38.7041</v>
+        <v>0</v>
       </c>
     </row>
     <row r="123" ht="14" customHeight="1">
@@ -1684,7 +1684,7 @@
         </is>
       </c>
       <c r="B123" s="7" t="n">
-        <v>40.2841</v>
+        <v>0</v>
       </c>
     </row>
     <row r="124" ht="14" customHeight="1">
@@ -1694,7 +1694,7 @@
         </is>
       </c>
       <c r="B124" s="7" t="n">
-        <v>40.2269</v>
+        <v>0</v>
       </c>
     </row>
     <row r="125" ht="14" customHeight="1">
@@ -1704,7 +1704,7 @@
         </is>
       </c>
       <c r="B125" s="7" t="n">
-        <v>40.653</v>
+        <v>0</v>
       </c>
     </row>
     <row r="126" ht="14" customHeight="1">
@@ -1984,7 +1984,7 @@
         <v>833.3333</v>
       </c>
       <c r="C3" t="n">
-        <v>6336</v>
+        <v>6365.8412</v>
       </c>
       <c r="D3" s="6" t="inlineStr">
         <is>
@@ -2002,10 +2002,10 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>4711.1111</v>
+        <v>4787.9643</v>
       </c>
       <c r="C4" t="n">
-        <v>1683</v>
+        <v>1702.997</v>
       </c>
     </row>
     <row r="5" ht="14" customFormat="1" customHeight="1" s="5">
@@ -2015,10 +2015,10 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>5288.8889</v>
+        <v>5286.0352</v>
       </c>
       <c r="C5" t="n">
-        <v>81</v>
+        <v>91.1014</v>
       </c>
     </row>
     <row r="6" ht="14" customFormat="1" customHeight="1" s="5">
@@ -2031,7 +2031,7 @@
         <v>0</v>
       </c>
       <c r="C6" t="n">
-        <v>5940</v>
+        <v>5780.1319</v>
       </c>
     </row>
     <row r="7" ht="14" customFormat="1" customHeight="1" s="5">
@@ -2044,7 +2044,7 @@
         <v>5333.3333</v>
       </c>
       <c r="C7" t="n">
-        <v>2700</v>
+        <v>2859.8681</v>
       </c>
     </row>
   </sheetData>

</xml_diff>